<commit_message>
Use source lists for applicants, project types and support types
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHwNN6RfVzTYVCS9bRLUAz
</commit_message>
<xml_diff>
--- a/entregables/Herramienta_seleccion_proyectos_FEAC_BCS.xlsx
+++ b/entregables/Herramienta_seleccion_proyectos_FEAC_BCS.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="285">
   <si>
     <t xml:space="preserve">Guía para seleccionar los proyectos que financia el Fondo</t>
   </si>
@@ -564,103 +564,157 @@
     <t xml:space="preserve">El que fije la Comisión</t>
   </si>
   <si>
-    <t xml:space="preserve">Listas de referencia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quién puede solicitar: sujetos públicos (de los tres órdenes de gobierno) y privados (comerciales y no comerciales). El tipo de apoyo y la forma de entregarlo deben ser coherentes con el objeto y el marco de actuación de cada proponente.</t>
+    <t xml:space="preserve">Quién puede solicitar, tipo de proyecto y tipo de apoyo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tomado del documento «Criterios de elegibilidad de proyectos». Son tres listas independientes. El tipo de apoyo y la forma de entregarlo deben ser coherentes con el objeto y las facultades de cada solicitante.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quién puede solicitar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Públicos (federal, estatal y municipal)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dependencias y órganos desconcentrados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Municipios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paraestatales, empresas de participación estatal y fideicomisos públicos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Privados comerciales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Empresas, desarrolladores inmobiliarios, proveedores gubernamentales, constructores, inversionistas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Privados no comerciales</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sociedad civil, ONG, academia, instituciones técnicas especializadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En la hoja Evaluación se elige una de estas opciones:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Público: dependencia u órgano desconcentrado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Público: municipio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Público: paraestatal, empresa de participación estatal o fideicomiso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Privado comercial: empresa, desarrollador, proveedor, constructor o inversionista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Privado no comercial: sociedad civil u ONG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Privado no comercial: academia o institución técnica</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de proyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estudios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evaluaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estrategias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Obras</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diseño</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inversión</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Procesos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financiamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administración</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intervención</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recomendaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Otros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de apoyo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financiero: Préstamo o cofinanciamiento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financiero: Aportación a fondo perdido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financiero: Inversión de capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financiero: Garantía</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Financiero: Subvención o subsidio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No financiero: Asesoría y capacitación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No financiero: Realización de estudios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No financiero: Vinculación con otras instituciones, fondeadores o especialistas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Evaluación de proyectos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escriba solo en las celdas amarillas. Lo gris se calcula solo. Los requisitos, criterios y niveles completos están en la hoja «Guía».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paso 1 · Requisitos mínimos (Sí / No)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paso 2 · Criterios de calificación (1 · 2 · 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proyecto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proponente</t>
   </si>
   <si>
     <t xml:space="preserve">Tipo de proponente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo de proyecto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo de apoyo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gobierno del Estado (dependencia u órgano desconcentrado)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estudio, plan o evaluación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Financiero: aportación a fondo perdido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Municipio</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Programa, estrategia o acción</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Financiero: cofinanciamiento</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paraestatal o fideicomiso público</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Obra o infraestructura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Financiero: préstamo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sociedad civil (OSC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diseño o proyecto ejecutivo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Financiero: garantía</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comunitaria o ejidal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capacitación o educación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No financiero: asesoría y capacitación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Academia o institución técnica</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Investigación o innovación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No financiero: realización de estudios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Empresa o desarrollador</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Otro</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No financiero: vinculación con fondeadores o especialistas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Evaluación de proyectos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Escriba solo en las celdas amarillas. Lo gris se calcula solo. Los requisitos, criterios y niveles completos están en la hoja «Guía».</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paso 1 · Requisitos mínimos (Sí / No)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paso 2 · Criterios de calificación (1 · 2 · 3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proyecto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proponente</t>
   </si>
   <si>
     <t xml:space="preserve">Tema (fracción)</t>
@@ -1388,7 +1442,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G68"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -2093,95 +2147,216 @@
         <v>181</v>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="5" t="s">
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="B61" s="5" t="s">
+      <c r="B62" s="5"/>
+    </row>
+    <row r="63" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="B63" s="8" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="8" t="s">
+    <row r="64" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="B64" s="8" t="s">
         <v>185</v>
       </c>
-      <c r="B62" s="8" t="s">
+    </row>
+    <row r="65" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="B65" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="C62" s="8" t="s">
+    </row>
+    <row r="66" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="7" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="8" t="s">
+      <c r="B66" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="B63" s="8" t="s">
+    </row>
+    <row r="67" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="C63" s="8" t="s">
+      <c r="B67" s="8" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="8" t="s">
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B64" s="8" t="s">
+    </row>
+    <row r="69" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="C64" s="8" t="s">
+    </row>
+    <row r="70" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="8" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="8" t="s">
+    <row r="71" customFormat="false" ht="128.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="B65" s="8" t="s">
+    </row>
+    <row r="72" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="C65" s="8" t="s">
+    </row>
+    <row r="73" customFormat="false" ht="90.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="8" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="8" t="s">
+    <row r="74" customFormat="false" ht="102.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="B66" s="8" t="s">
+    </row>
+    <row r="76" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="C66" s="8" t="s">
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="8" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="8" t="s">
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="B67" s="8" t="s">
+    </row>
+    <row r="79" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="C67" s="8" t="s">
+    </row>
+    <row r="80" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="8" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="8" t="s">
+    <row r="81" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="B68" s="8" t="s">
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="C68" s="8" t="s">
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="8" t="s">
         <v>205</v>
       </c>
     </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="8" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="8" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="8" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="8" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="8" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="8" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="8" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="8" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="5" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="8" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="95" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A95" s="8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A96" s="8" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A97" s="8" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="64.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A98" s="8" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A99" s="8" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="77.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="8" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="153.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A101" s="8" t="s">
+        <v>222</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A62:B62"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2219,17 +2394,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>206</v>
+        <v>223</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>207</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="I4" s="10" t="s">
-        <v>208</v>
+        <v>225</v>
       </c>
       <c r="J4" s="10"/>
       <c r="K4" s="10"/>
@@ -2239,7 +2414,7 @@
       <c r="O4" s="10"/>
       <c r="P4" s="10"/>
       <c r="Q4" s="10" t="s">
-        <v>209</v>
+        <v>226</v>
       </c>
       <c r="R4" s="10"/>
       <c r="S4" s="10"/>
@@ -2253,91 +2428,91 @@
     </row>
     <row r="5" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>182</v>
+        <v>230</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>183</v>
+        <v>198</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>184</v>
+        <v>214</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>213</v>
+        <v>231</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>214</v>
+        <v>232</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>215</v>
+        <v>233</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>216</v>
+        <v>234</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>217</v>
+        <v>235</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>218</v>
+        <v>236</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>219</v>
+        <v>237</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>220</v>
+        <v>238</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="P5" s="5" t="s">
-        <v>222</v>
+        <v>240</v>
       </c>
       <c r="Q5" s="5" t="s">
-        <v>223</v>
+        <v>241</v>
       </c>
       <c r="R5" s="5" t="s">
-        <v>224</v>
+        <v>242</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>225</v>
+        <v>243</v>
       </c>
       <c r="T5" s="5" t="s">
-        <v>226</v>
+        <v>244</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>227</v>
+        <v>245</v>
       </c>
       <c r="V5" s="5" t="s">
-        <v>228</v>
+        <v>246</v>
       </c>
       <c r="W5" s="5" t="s">
-        <v>229</v>
+        <v>247</v>
       </c>
       <c r="X5" s="5" t="s">
-        <v>230</v>
+        <v>248</v>
       </c>
       <c r="Y5" s="5" t="s">
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="Z5" s="5" t="s">
         <v>97</v>
       </c>
       <c r="AA5" s="5" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
       <c r="AB5" s="5" t="s">
-        <v>233</v>
+        <v>251</v>
       </c>
       <c r="AC5" s="5" t="s">
-        <v>234</v>
+        <v>252</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2386,22 +2561,22 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>235</v>
+        <v>253</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>237</v>
+        <v>255</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="F7" s="12" t="s">
-        <v>187</v>
+        <v>216</v>
       </c>
       <c r="G7" s="12" t="s">
         <v>128</v>
@@ -2410,22 +2585,22 @@
         <v>2500000</v>
       </c>
       <c r="I7" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="J7" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="K7" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="L7" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="M7" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="N7" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="O7" s="15" t="str">
         <f aca="false">IF(A7="","",IF(COUNTIF(I7:N7,"No")&gt;0,"No",IF(COUNTIF(I7:N7,"Sí")=6,"Sí","Falta información")))</f>
@@ -2472,7 +2647,7 @@
         <v>1</v>
       </c>
       <c r="AB7" s="12" t="s">
-        <v>239</v>
+        <v>257</v>
       </c>
       <c r="AC7" s="15" t="n">
         <f aca="false">IF(A7="","",IF(Y7&lt;&gt;"",Y7*10000+Q7*100+R7-ROW()/1000,-ROW()))</f>
@@ -2481,22 +2656,22 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>240</v>
+        <v>258</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>241</v>
+        <v>259</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>242</v>
+        <v>260</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>190</v>
+        <v>215</v>
       </c>
       <c r="G8" s="12" t="s">
         <v>136</v>
@@ -2505,22 +2680,22 @@
         <v>4000000</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="K8" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="L8" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="M8" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="N8" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="O8" s="15" t="str">
         <f aca="false">IF(A8="","",IF(COUNTIF(I8:N8,"No")&gt;0,"No",IF(COUNTIF(I8:N8,"Sí")=6,"Sí","Falta información")))</f>
@@ -2567,7 +2742,7 @@
         <v>2</v>
       </c>
       <c r="AB8" s="12" t="s">
-        <v>243</v>
+        <v>261</v>
       </c>
       <c r="AC8" s="15" t="n">
         <f aca="false">IF(A8="","",IF(Y8&lt;&gt;"",Y8*10000+Q8*100+R8-ROW()/1000,-ROW()))</f>
@@ -2576,22 +2751,22 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>245</v>
+        <v>263</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>246</v>
+        <v>264</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>192</v>
+        <v>205</v>
       </c>
       <c r="F9" s="12" t="s">
-        <v>190</v>
+        <v>215</v>
       </c>
       <c r="G9" s="12" t="s">
         <v>148</v>
@@ -2600,22 +2775,22 @@
         <v>3000000</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="O9" s="15" t="str">
         <f aca="false">IF(A9="","",IF(COUNTIF(I9:N9,"No")&gt;0,"No",IF(COUNTIF(I9:N9,"Sí")=6,"Sí","Falta información")))</f>
@@ -2662,7 +2837,7 @@
         <v>3</v>
       </c>
       <c r="AB9" s="12" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
       <c r="AC9" s="15" t="n">
         <f aca="false">IF(A9="","",IF(Y9&lt;&gt;"",Y9*10000+Q9*100+R9-ROW()/1000,-ROW()))</f>
@@ -2671,22 +2846,22 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>249</v>
+        <v>267</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>250</v>
+        <v>268</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>187</v>
+        <v>216</v>
       </c>
       <c r="G10" s="12" t="s">
         <v>152</v>
@@ -2695,22 +2870,22 @@
         <v>600000</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>251</v>
+        <v>269</v>
       </c>
       <c r="K10" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="L10" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="M10" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="N10" s="14" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="O10" s="15" t="str">
         <f aca="false">IF(A10="","",IF(COUNTIF(I10:N10,"No")&gt;0,"No",IF(COUNTIF(I10:N10,"Sí")=6,"Sí","Falta información")))</f>
@@ -2741,7 +2916,7 @@
         <v/>
       </c>
       <c r="AB10" s="12" t="s">
-        <v>252</v>
+        <v>270</v>
       </c>
       <c r="AC10" s="15" t="n">
         <f aca="false">IF(A10="","",IF(Y10&lt;&gt;"",Y10*10000+Q10*100+R10-ROW()/1000,-ROW()))</f>
@@ -5043,15 +5218,15 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D7:D56" type="list">
-      <formula1>Guía!$A$62:$A$68</formula1>
+      <formula1>Guía!$A$69:$A$74</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E7:E56" type="list">
-      <formula1>Guía!$B$62:$B$68</formula1>
+      <formula1>Guía!$A$77:$A$91</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F7:F56" type="list">
-      <formula1>Guía!$C$62:$C$68</formula1>
+      <formula1>Guía!$A$94:$A$101</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -5088,17 +5263,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>253</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>254</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
       <c r="C4" s="19" t="n">
         <f aca="false">COUNTIF(Evaluación!$A$7:$A$56,"?*")</f>
@@ -5107,7 +5282,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>256</v>
+        <v>274</v>
       </c>
       <c r="C5" s="19" t="n">
         <f aca="false">COUNTIF(Evaluación!$O$7:$O$56,"Sí")</f>
@@ -5116,7 +5291,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>257</v>
+        <v>275</v>
       </c>
       <c r="C6" s="19" t="n">
         <f aca="false">COUNTIF(Evaluación!$O$7:$O$56,"No")</f>
@@ -5125,7 +5300,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>258</v>
+        <v>276</v>
       </c>
       <c r="C7" s="19" t="n">
         <f aca="false">COUNTIF(Evaluación!$O$7:$O$56,"Falta información")</f>
@@ -5134,7 +5309,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>259</v>
+        <v>277</v>
       </c>
       <c r="C8" s="19" t="n">
         <f aca="false">COUNTIF(Evaluación!$Z$7:$Z$56,"Alta")</f>
@@ -5143,7 +5318,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
       <c r="C9" s="19" t="n">
         <f aca="false">COUNTIF(Evaluación!$Z$7:$Z$56,"Media")</f>
@@ -5152,7 +5327,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
       <c r="C10" s="19" t="n">
         <f aca="false">COUNTIF(Evaluación!$Z$7:$Z$56,"Baja")</f>
@@ -5161,7 +5336,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>262</v>
+        <v>280</v>
       </c>
       <c r="C11" s="20" t="n">
         <f aca="false">SUMIF(Evaluación!$Z$7:$Z$56,"Alta",Evaluación!$H$7:$H$56)</f>
@@ -5170,22 +5345,22 @@
     </row>
     <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>232</v>
+        <v>250</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>263</v>
+        <v>281</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>113</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>264</v>
+        <v>282</v>
       </c>
       <c r="G14" s="5" t="s">
         <v>98</v>
@@ -5194,13 +5369,13 @@
         <v>97</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>221</v>
+        <v>239</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>266</v>
+        <v>284</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5218,7 +5393,7 @@
       </c>
       <c r="D15" s="15" t="str">
         <f aca="false">IF($K15="","",IF(INDEX(Evaluación!$D$7:$D$56,$K15)="","",INDEX(Evaluación!$D$7:$D$56,$K15)))</f>
-        <v>Sociedad civil (OSC)</v>
+        <v>Privado no comercial: sociedad civil u ONG</v>
       </c>
       <c r="E15" s="15" t="str">
         <f aca="false">IF($K15="","",IF(INDEX(Evaluación!$G$7:$G$56,$K15)="","",INDEX(Evaluación!$G$7:$G$56,$K15)))</f>
@@ -5264,7 +5439,7 @@
       </c>
       <c r="D16" s="15" t="str">
         <f aca="false">IF($K16="","",IF(INDEX(Evaluación!$D$7:$D$56,$K16)="","",INDEX(Evaluación!$D$7:$D$56,$K16)))</f>
-        <v>Gobierno del Estado (dependencia u órgano desconcentrado)</v>
+        <v>Público: dependencia u órgano desconcentrado</v>
       </c>
       <c r="E16" s="15" t="str">
         <f aca="false">IF($K16="","",IF(INDEX(Evaluación!$G$7:$G$56,$K16)="","",INDEX(Evaluación!$G$7:$G$56,$K16)))</f>
@@ -5310,7 +5485,7 @@
       </c>
       <c r="D17" s="15" t="str">
         <f aca="false">IF($K17="","",IF(INDEX(Evaluación!$D$7:$D$56,$K17)="","",INDEX(Evaluación!$D$7:$D$56,$K17)))</f>
-        <v>Municipio</v>
+        <v>Público: municipio</v>
       </c>
       <c r="E17" s="15" t="str">
         <f aca="false">IF($K17="","",IF(INDEX(Evaluación!$G$7:$G$56,$K17)="","",INDEX(Evaluación!$G$7:$G$56,$K17)))</f>
@@ -5356,7 +5531,7 @@
       </c>
       <c r="D18" s="15" t="str">
         <f aca="false">IF($K18="","",IF(INDEX(Evaluación!$D$7:$D$56,$K18)="","",INDEX(Evaluación!$D$7:$D$56,$K18)))</f>
-        <v>Sociedad civil (OSC)</v>
+        <v>Privado no comercial: sociedad civil u ONG</v>
       </c>
       <c r="E18" s="15" t="str">
         <f aca="false">IF($K18="","",IF(INDEX(Evaluación!$G$7:$G$56,$K18)="","",INDEX(Evaluación!$G$7:$G$56,$K18)))</f>

</xml_diff>

<commit_message>
Ground guide only in the fund decree and use promovente
Remove references to source documents, name the evaluation body as the
decree's Subcomité Técnico Especializado, and replace annex B with the
decree articles each part of the guide applies.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VHwNN6RfVzTYVCS9bRLUAz
</commit_message>
<xml_diff>
--- a/entregables/Herramienta_seleccion_proyectos_FEAC_BCS.xlsx
+++ b/entregables/Herramienta_seleccion_proyectos_FEAC_BCS.xlsx
@@ -22,12 +22,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="337">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="338">
   <si>
     <t xml:space="preserve">Guía para seleccionar los proyectos que financia el Fondo</t>
   </si>
   <si>
-    <t xml:space="preserve">Fondo Estatal Ambiental y Climático de Baja California Sur (FEAC BCS). Se aplica igual a proyectos del Estado, de los municipios y de la sociedad civil. Basada en los Criterios de elegibilidad de proyectos y en el Decreto del Fondo.</t>
+    <t xml:space="preserve">Fondo Estatal Ambiental y Climático de Baja California Sur (FEAC BCS). Se aplica igual a proyectos del Estado, de los municipios y de la sociedad civil. Con fundamento en el Decreto del Fondo.</t>
   </si>
   <si>
     <t xml:space="preserve">Cómo usar esta herramienta</t>
@@ -42,7 +42,7 @@
     <t xml:space="preserve">3. Paso 2 · Criterios de calificación: si puede participar, califique los 8 criterios de 1 a 3 con la tabla de abajo. Los puntos y la prioridad se calculan solos.</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Paso 3: la hoja «Ranking» ordena los proyectos por puntos. El Comité de Evaluación y Seguimiento propone y el Comité Técnico decide con base en ese orden y en el presupuesto.</t>
+    <t xml:space="preserve">4. Paso 3: la hoja «Ranking» ordena los proyectos por puntos. El Subcomité Técnico Especializado propone y el Comité Técnico decide con base en ese orden y en el presupuesto.</t>
   </si>
   <si>
     <t xml:space="preserve">Cada calificación del Paso 2 debe justificarse en la columna «Justificación»; si falta, la hoja lo marca en «Alertas». Las filas EJ-1 a EJ-5 son ejemplos; bórrelas antes de evaluar proyectos reales.</t>
@@ -75,16 +75,16 @@
     <t xml:space="preserve">Calibración de evaluadores</t>
   </si>
   <si>
-    <t xml:space="preserve">Antes de la primera convocatoria, y cuando entren evaluadores nuevos, el Comité de Evaluación califica en conjunto 2 o 3 proyectos de prueba y acuerda cómo interpretar cada nivel.</t>
+    <t xml:space="preserve">Antes de la primera convocatoria, y cuando entren evaluadores nuevos, el Subcomité Técnico Especializado califica en conjunto 2 o 3 proyectos de prueba y acuerda cómo interpretar cada nivel.</t>
   </si>
   <si>
     <t xml:space="preserve">Fichas técnicas por tema</t>
   </si>
   <si>
-    <t xml:space="preserve">El Comité de Evaluación y Seguimiento elabora, y el Comité Técnico aprueba, una ficha por tema que dice qué es un impacto alto, medio o bajo y con qué se compara. Se empieza por los temas con más demanda y se completan conforme lleguen proyectos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Formato de ficha técnica por tema (lo llena el Comité de Evaluación y Seguimiento)</t>
+    <t xml:space="preserve">El Subcomité Técnico Especializado elabora, y el Comité Técnico aprueba, una ficha por tema que dice qué es un impacto alto, medio o bajo y con qué se compara. Se empieza por los temas con más demanda y se completan conforme lleguen proyectos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Formato de ficha técnica por tema (lo llena el Subcomité Técnico Especializado)</t>
   </si>
   <si>
     <t xml:space="preserve">Campo</t>
@@ -120,7 +120,7 @@
     <t xml:space="preserve">Fuentes de referencia</t>
   </si>
   <si>
-    <t xml:space="preserve">Estudios, diagnósticos o sistemas que respaldan los valores (por ejemplo, el Sistema de Priorización de SbN de Forest Trends para agua)</t>
+    <t xml:space="preserve">Estudios, diagnósticos o sistemas que respaldan los valores (por ejemplo, diagnósticos estatales, programas de manejo o estudios especializados)</t>
   </si>
   <si>
     <t xml:space="preserve">Responsable y fecha</t>
@@ -129,7 +129,7 @@
     <t xml:space="preserve">Quién la elaboró, cuándo la aprobó el Comité Técnico y cuándo se revisa</t>
   </si>
   <si>
-    <t xml:space="preserve">Mientras un tema no tenga ficha, el evaluador califica el Impacto comparando la meta del proyecto con su línea base y con el diagnóstico del problema que presenta el proponente, y lo deja escrito en la justificación.</t>
+    <t xml:space="preserve">Mientras un tema no tenga ficha, el evaluador califica el Impacto comparando la meta del proyecto con su línea base y con el diagnóstico del problema que presenta el promovente, y lo deja escrito en la justificación.</t>
   </si>
   <si>
     <t xml:space="preserve">Además, el Comité Técnico puede fijar prioridades en cada convocatoria, por ejemplo reservar una parte del presupuesto para agua dada la escasez hídrica del Estado, sin cambiar los criterios de calificación.</t>
@@ -222,10 +222,10 @@
     <t xml:space="preserve">Análisis de impactos; permisos o plan para tramitarlos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Proponente en regla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Que el proponente tenga su documentación en orden, pida un monto dentro del rango y no reciba otro apoyo para lo mismo.</t>
+    <t xml:space="preserve">Promovente en regla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Que el promovente tenga su documentación en orden, pida un monto dentro del rango y no reciba otro apoyo para lo mismo.</t>
   </si>
   <si>
     <t xml:space="preserve">Entrega el soporte documental de su situación legal, financiera y fiscal; el monto está dentro del rango; declara que no tiene otro apoyo para lo mismo y que el proyecto no está ya hecho; y establece cómo informará sus avances (al menos cada trimestre).</t>
@@ -303,13 +303,13 @@
     <t xml:space="preserve">Factibilidad</t>
   </si>
   <si>
-    <t xml:space="preserve">Viabilidad técnica, administrativa y legal: madurez del proyecto, experiencia del proponente y manejo de riesgos y obstáculos.</t>
+    <t xml:space="preserve">Viabilidad técnica, administrativa y legal: madurez del proyecto, experiencia del promovente y manejo de riesgos y obstáculos.</t>
   </si>
   <si>
     <t xml:space="preserve">x1</t>
   </si>
   <si>
-    <t xml:space="preserve">Proyecto ejecutivo o muy avanzado; el proponente ya hizo proyectos parecidos; los riesgos y obstáculos están identificados y tienen solución.</t>
+    <t xml:space="preserve">Proyecto ejecutivo o muy avanzado; el promovente ya hizo proyectos parecidos; los riesgos y obstáculos están identificados y tienen solución.</t>
   </si>
   <si>
     <t xml:space="preserve">Anteproyecto; experiencia parcial; riesgos identificados sin soluciones claras.</t>
@@ -693,7 +693,7 @@
     <t xml:space="preserve">Quién puede solicitar, tipo de proyecto y tipo de apoyo</t>
   </si>
   <si>
-    <t xml:space="preserve">Tomado del documento «Criterios de elegibilidad de proyectos». Son tres listas independientes. El tipo de apoyo y la forma de entregarlo deben ser coherentes con el objeto y las facultades de cada solicitante.</t>
+    <t xml:space="preserve">Son tres listas independientes. El tipo de apoyo y la forma de entregarlo deben ser coherentes con el objeto y las facultades de cada solicitante.</t>
   </si>
   <si>
     <t xml:space="preserve">Quién puede solicitar</t>
@@ -837,10 +837,10 @@
     <t xml:space="preserve">Proyecto</t>
   </si>
   <si>
-    <t xml:space="preserve">Proponente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tipo de proponente</t>
+    <t xml:space="preserve">Promovente</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo de promovente</t>
   </si>
   <si>
     <t xml:space="preserve">Tema (fracción)</t>
@@ -864,7 +864,7 @@
     <t xml:space="preserve">R5. No causa daño ambiental</t>
   </si>
   <si>
-    <t xml:space="preserve">R6. Proponente en regla</t>
+    <t xml:space="preserve">R6. Promovente en regla</t>
   </si>
   <si>
     <t xml:space="preserve">¿Puede participar?</t>
@@ -933,7 +933,7 @@
     <t xml:space="preserve">Sí</t>
   </si>
   <si>
-    <t xml:space="preserve">Agua y SbN (referencia: Forest Trends)</t>
+    <t xml:space="preserve">Ficha IV · Conservación de ecosistemas (ejemplo)</t>
   </si>
   <si>
     <t xml:space="preserve">Ejemplo. Impacto 3: restaura 45 ha de manglar en una laguna con pérdida documentada. Vulnerabilidad 3: comunidad pesquera costera en zona de riesgo por huracanes. Sostenibilidad 2: hay cofinanciamiento, pero sin acuerdo de mantenimiento.</t>
@@ -985,6 +985,9 @@
   </si>
   <si>
     <t xml:space="preserve">Parque lineal con captación de lluvia (ejemplo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ficha XII · Infraestructura verde (ejemplo)</t>
   </si>
   <si>
     <t xml:space="preserve">Ejemplo. Factibilidad 3: proyecto ejecutivo. Costo-efectividad 1: no calcula costo por m3 captado. Sostenibilidad 1: nadie se compromete a mantenerlo. Candidato a fortalecimiento.</t>
@@ -3529,10 +3532,10 @@
         <v>Costo-efectividad; Sostenibilidad;</v>
       </c>
       <c r="AD11" s="15" t="s">
-        <v>303</v>
+        <v>321</v>
       </c>
       <c r="AE11" s="15" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="AF11" s="18" t="str">
         <f aca="false">IF(Y11="","",IF(AE11="","Falta justificación",""))</f>
@@ -6433,17 +6436,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C4" s="22" t="n">
         <f aca="false">COUNTIF(Evaluación!$A$7:$A$56,"?*")</f>
@@ -6452,7 +6455,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C5" s="22" t="n">
         <f aca="false">COUNTIF(Evaluación!$O$7:$O$56,"Sí*")</f>
@@ -6461,7 +6464,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="C6" s="22" t="n">
         <f aca="false">COUNTIF(Evaluación!$AB$7:$AB$56,"Candidato*")</f>
@@ -6470,7 +6473,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C7" s="22" t="n">
         <f aca="false">COUNTIF(Evaluación!$AF$7:$AF$56,"Falta*")</f>
@@ -6479,7 +6482,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C8" s="22" t="n">
         <f aca="false">COUNTIF(Evaluación!$O$7:$O$56,"No")</f>
@@ -6488,7 +6491,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C9" s="22" t="n">
         <f aca="false">COUNTIF(Evaluación!$O$7:$O$56,"Falta información")</f>
@@ -6497,7 +6500,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C10" s="22" t="n">
         <f aca="false">COUNTIF(Evaluación!$Z$7:$Z$56,"Alta")</f>
@@ -6506,7 +6509,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C11" s="22" t="n">
         <f aca="false">COUNTIF(Evaluación!$Z$7:$Z$56,"Media")</f>
@@ -6515,7 +6518,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C12" s="22" t="n">
         <f aca="false">COUNTIF(Evaluación!$Z$7:$Z$56,"Baja")</f>
@@ -6524,7 +6527,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C13" s="23" t="n">
         <f aca="false">SUMIF(Evaluación!$Z$7:$Z$56,"Alta",Evaluación!$H$7:$H$56)</f>
@@ -6548,7 +6551,7 @@
         <v>155</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G15" s="6" t="s">
         <v>140</v>
@@ -6560,13 +6563,13 @@
         <v>281</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K15" s="6" t="s">
         <v>293</v>
       </c>
       <c r="L15" s="6" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>